<commit_message>
updated IBM Synth Graph Evaluation
</commit_message>
<xml_diff>
--- a/evaluation/IbmSynth/results/evaluation_graph.xlsx
+++ b/evaluation/IbmSynth/results/evaluation_graph.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,10 +436,15 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>NetSimile</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>DeltaCon0</t>
         </is>
@@ -451,11 +456,32 @@
           <t>DOPPELGANGER</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>distance</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>30.55801542549026</v>
       </c>
-      <c r="C2" t="n">
-        <v>179.5145787121959</v>
+      <c r="D2" t="n">
+        <v>179.4850357505663</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DOPPELGANGER</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>72.72203950474218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>